<commit_message>
inflections: new inflections from commentaries
</commit_message>
<xml_diff>
--- a/db/inflections/inflection_templates.xlsx
+++ b/db/inflections/inflection_templates.xlsx
@@ -2619,6 +2619,7 @@
   </si>
   <si>
     <t xml:space="preserve">tayi
+tayī
 tvāyi</t>
   </si>
   <si>
@@ -3473,6 +3474,7 @@
     <t xml:space="preserve">assaṃ
 imāyaṃ
 imissaṃ
+imissāya
 imissāyaṃ</t>
   </si>
   <si>
@@ -44042,7 +44044,7 @@
       </c>
       <c r="DK39" s="47"/>
     </row>
-    <row r="40" customFormat="false" ht="56.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="21" t="s">
         <v>519</v>
       </c>

</xml_diff>